<commit_message>
ECLE naming, harmonised palette and category order
The category "cancer-like endometriosis (CLE)" is now "Endometriosis CLE"
(short label ECLE; endometriosis with cancer-like PD-L1 expression). Notebook 20
renamed 20_DGE_Bulk_ECLE; inputs recoded to the new category name; one colour
palette for all figures; categories shown in the order SE, ECLE, AE, CCC, EC;
reproducible volcano labels. Results unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/DATA_INPUT/IHC_public.xlsx
+++ b/DATA_INPUT/IHC_public.xlsx
@@ -1,136 +1,143 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <workbookPr date1904="false"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Spoiler\SPOILER_Submission\DATA_INPUT\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AD485D0-C8D5-4BE0-940B-31F2835462CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" firstSheet="0" activeTab="0"/>
+    <workbookView xWindow="140" yWindow="0" windowWidth="18380" windowHeight="15280" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="IHC" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="IHC" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
-  <si>
-    <t xml:space="preserve">Patient</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Category</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MLH1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PMS2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MSH2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MSH6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MMR status</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ER</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">β-catenin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pt_05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Simple endometriosis</t>
-  </si>
-  <si>
-    <t xml:space="preserve">+</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MMRp</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Membranous</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pt_04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pt_03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cancer-like endometriosis</t>
-  </si>
-  <si>
-    <t xml:space="preserve">−</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pt_02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pt_13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pt_14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Indet.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pt_08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Atypical endometriosis</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MMRd</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pt_07</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Predominantly membranous, focally cytoplasmic</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pt_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Clear cell carcinoma</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pt_09</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pt_10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pt_06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Endometrioid carcinoma</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pt_11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Membranous and nuclear</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pt_12</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="37">
+  <si>
+    <t>Patient</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>MLH1</t>
+  </si>
+  <si>
+    <t>PMS2</t>
+  </si>
+  <si>
+    <t>MSH2</t>
+  </si>
+  <si>
+    <t>MSH6</t>
+  </si>
+  <si>
+    <t>MMR status</t>
+  </si>
+  <si>
+    <t>ER</t>
+  </si>
+  <si>
+    <t>PR</t>
+  </si>
+  <si>
+    <t>β-catenin</t>
+  </si>
+  <si>
+    <t>Pt_05</t>
+  </si>
+  <si>
+    <t>Simple endometriosis</t>
+  </si>
+  <si>
+    <t>+</t>
+  </si>
+  <si>
+    <t>MMRp</t>
+  </si>
+  <si>
+    <t>Membranous</t>
+  </si>
+  <si>
+    <t>Pt_04</t>
+  </si>
+  <si>
+    <t>Pt_03</t>
+  </si>
+  <si>
+    <t>−</t>
+  </si>
+  <si>
+    <t>Pt_02</t>
+  </si>
+  <si>
+    <t>Pt_13</t>
+  </si>
+  <si>
+    <t>Pt_14</t>
+  </si>
+  <si>
+    <t>Indet.</t>
+  </si>
+  <si>
+    <t>Pt_08</t>
+  </si>
+  <si>
+    <t>Atypical endometriosis</t>
+  </si>
+  <si>
+    <t>MMRd</t>
+  </si>
+  <si>
+    <t>Pt_07</t>
+  </si>
+  <si>
+    <t>Predominantly membranous, focally cytoplasmic</t>
+  </si>
+  <si>
+    <t>Pt_01</t>
+  </si>
+  <si>
+    <t>Clear cell carcinoma</t>
+  </si>
+  <si>
+    <t>Pt_09</t>
+  </si>
+  <si>
+    <t>Pt_10</t>
+  </si>
+  <si>
+    <t>Pt_06</t>
+  </si>
+  <si>
+    <t>Endometrioid carcinoma</t>
+  </si>
+  <si>
+    <t>Pt_11</t>
+  </si>
+  <si>
+    <t>Membranous and nuclear</t>
+  </si>
+  <si>
+    <t>Pt_12</t>
+  </si>
+  <si>
+    <t>Endometriosis CLE</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -166,6 +173,15 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -447,11 +463,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:J15"/>
+  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -483,7 +499,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -515,7 +531,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -547,12 +563,12 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>16</v>
       </c>
       <c r="B4" t="s">
-        <v>17</v>
+        <v>36</v>
       </c>
       <c r="C4" t="s">
         <v>12</v>
@@ -573,18 +589,18 @@
         <v>12</v>
       </c>
       <c r="I4" t="s">
+        <v>17</v>
+      </c>
+      <c r="J4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
         <v>18</v>
       </c>
-      <c r="J4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="s">
-        <v>19</v>
-      </c>
       <c r="B5" t="s">
-        <v>17</v>
+        <v>36</v>
       </c>
       <c r="C5" t="s">
         <v>12</v>
@@ -605,18 +621,18 @@
         <v>12</v>
       </c>
       <c r="I5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J5" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B6" t="s">
-        <v>17</v>
+        <v>36</v>
       </c>
       <c r="C6" t="s">
         <v>12</v>
@@ -637,82 +653,82 @@
         <v>12</v>
       </c>
       <c r="I6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J6" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B7" t="s">
-        <v>17</v>
+        <v>36</v>
       </c>
       <c r="C7" t="s">
+        <v>21</v>
+      </c>
+      <c r="D7" t="s">
+        <v>21</v>
+      </c>
+      <c r="E7" t="s">
+        <v>21</v>
+      </c>
+      <c r="F7" t="s">
+        <v>21</v>
+      </c>
+      <c r="G7" t="s">
+        <v>21</v>
+      </c>
+      <c r="H7" t="s">
+        <v>12</v>
+      </c>
+      <c r="I7" t="s">
+        <v>17</v>
+      </c>
+      <c r="J7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
         <v>22</v>
       </c>
-      <c r="D7" t="s">
-        <v>22</v>
-      </c>
-      <c r="E7" t="s">
-        <v>22</v>
-      </c>
-      <c r="F7" t="s">
-        <v>22</v>
-      </c>
-      <c r="G7" t="s">
-        <v>22</v>
-      </c>
-      <c r="H7" t="s">
-        <v>12</v>
-      </c>
-      <c r="I7" t="s">
-        <v>18</v>
-      </c>
-      <c r="J7" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="s">
+      <c r="B8" t="s">
         <v>23</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C8" t="s">
+        <v>17</v>
+      </c>
+      <c r="D8" t="s">
+        <v>17</v>
+      </c>
+      <c r="E8" t="s">
+        <v>12</v>
+      </c>
+      <c r="F8" t="s">
+        <v>12</v>
+      </c>
+      <c r="G8" t="s">
         <v>24</v>
       </c>
-      <c r="C8" t="s">
-        <v>18</v>
-      </c>
-      <c r="D8" t="s">
-        <v>18</v>
-      </c>
-      <c r="E8" t="s">
-        <v>12</v>
-      </c>
-      <c r="F8" t="s">
-        <v>12</v>
-      </c>
-      <c r="G8" t="s">
+      <c r="H8" t="s">
+        <v>12</v>
+      </c>
+      <c r="I8" t="s">
+        <v>12</v>
+      </c>
+      <c r="J8" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
         <v>25</v>
       </c>
-      <c r="H8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I8" t="s">
-        <v>12</v>
-      </c>
-      <c r="J8" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="s">
-        <v>26</v>
-      </c>
       <c r="B9" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C9" t="s">
         <v>12</v>
@@ -736,47 +752,47 @@
         <v>12</v>
       </c>
       <c r="J9" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="s">
+      <c r="B10" t="s">
         <v>28</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
+        <v>12</v>
+      </c>
+      <c r="D10" t="s">
+        <v>21</v>
+      </c>
+      <c r="E10" t="s">
+        <v>21</v>
+      </c>
+      <c r="F10" t="s">
+        <v>21</v>
+      </c>
+      <c r="G10" t="s">
+        <v>21</v>
+      </c>
+      <c r="H10" t="s">
+        <v>17</v>
+      </c>
+      <c r="I10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J10" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
         <v>29</v>
       </c>
-      <c r="C10" t="s">
-        <v>12</v>
-      </c>
-      <c r="D10" t="s">
-        <v>22</v>
-      </c>
-      <c r="E10" t="s">
-        <v>22</v>
-      </c>
-      <c r="F10" t="s">
-        <v>22</v>
-      </c>
-      <c r="G10" t="s">
-        <v>22</v>
-      </c>
-      <c r="H10" t="s">
-        <v>18</v>
-      </c>
-      <c r="I10" t="s">
-        <v>18</v>
-      </c>
-      <c r="J10" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="s">
-        <v>30</v>
-      </c>
       <c r="B11" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C11" t="s">
         <v>12</v>
@@ -803,12 +819,12 @@
         <v>14</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C12" t="s">
         <v>12</v>
@@ -826,21 +842,21 @@
         <v>13</v>
       </c>
       <c r="H12" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I12" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J12" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
+        <v>31</v>
+      </c>
+      <c r="B13" t="s">
         <v>32</v>
-      </c>
-      <c r="B13" t="s">
-        <v>33</v>
       </c>
       <c r="C13" t="s">
         <v>12</v>
@@ -867,12 +883,12 @@
         <v>14</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B14" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C14" t="s">
         <v>12</v>
@@ -896,15 +912,15 @@
         <v>12</v>
       </c>
       <c r="J14" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="s">
-        <v>36</v>
-      </c>
       <c r="B15" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C15" t="s">
         <v>12</v>
@@ -916,16 +932,16 @@
         <v>12</v>
       </c>
       <c r="F15" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G15" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H15" t="s">
         <v>12</v>
       </c>
       <c r="I15" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J15" t="s">
         <v>14</v>
@@ -933,6 +949,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
</xml_diff>